<commit_message>
Add quicklinks blocks, improve cards functionality, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (10):
- blocks/cards/cards.css
- blocks/cards/cards.js
- blocks/quicklinks/quicklinks.css
- blocks/quicklinks/quicklinks.js
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/parsers/quicklinks.js
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/index.report.json
- tools/importer/transformers/verizon-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","hero"]</t>
+    <t>["quicklinks","hero","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","hero"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-03-19T21:22:52.281Z</t>
+    <t>2026-03-20T00:24:54.614Z</t>
   </si>
   <si>
     <t>Verizon: Wireless, Internet, TV and Phone Services | Official Site</t>

</xml_diff>